<commit_message>
perbaikan pada data anggota dan kartu anggota
</commit_message>
<xml_diff>
--- a/public/template/template_import_anggota.xlsx
+++ b/public/template/template_import_anggota.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felix\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACF4F7F-F96D-4885-AF36-EEA21A0D9443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB546415-008D-4389-8D21-6FA2AE1461BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F998C215-5626-4A2B-8EB0-329C20B518CF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{95ED1428-B8F2-4AD6-9B02-BC1551C2AD85}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,11 +34,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+  <si>
+    <t>nomor_anggota</t>
+  </si>
   <si>
     <t>nama_lengkap</t>
   </si>
   <si>
+    <t>tempat_lahir</t>
+  </si>
+  <si>
     <t>jenis_kelamin</t>
   </si>
   <si>
@@ -57,25 +63,34 @@
     <t>status</t>
   </si>
   <si>
-    <t>nomor_anggota</t>
-  </si>
-  <si>
-    <t>Budi Santoso</t>
+    <t>tanggal_lahir</t>
+  </si>
+  <si>
+    <t>SANGGAU LEDO</t>
+  </si>
+  <si>
+    <t>VII A</t>
+  </si>
+  <si>
+    <t>jl.mawar</t>
+  </si>
+  <si>
+    <t>aktif</t>
+  </si>
+  <si>
+    <t>FELLIX</t>
+  </si>
+  <si>
+    <t>24-08-2004</t>
+  </si>
+  <si>
+    <t>15-03-2025</t>
+  </si>
+  <si>
+    <t>AGT2025001</t>
   </si>
   <si>
     <t>L</t>
-  </si>
-  <si>
-    <t>VII A</t>
-  </si>
-  <si>
-    <t>Jl. Mawar</t>
-  </si>
-  <si>
-    <t>aktif</t>
-  </si>
-  <si>
-    <t>AGT2024001</t>
   </si>
 </sst>
 </file>
@@ -111,11 +126,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,33 +442,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E31B099-2E67-494F-A36A-F467D189D553}">
-  <dimension ref="A1:O2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C65485-1B00-4E24-82C0-B4EC565A52F1}">
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="16.5546875" customWidth="1"/>
-    <col min="5" max="5" width="16.77734375" customWidth="1"/>
-    <col min="6" max="6" width="16.6640625" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" customWidth="1"/>
-    <col min="8" max="8" width="10.88671875" customWidth="1"/>
-    <col min="15" max="15" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="4" max="5" width="13.77734375" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+    <col min="9" max="9" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -469,35 +480,44 @@
       <c r="H1" t="s">
         <v>6</v>
       </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2">
-        <v>8123456789</v>
-      </c>
-      <c r="G2" s="3">
-        <v>45483</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>